<commit_message>
Audit and fix slot placements and typos across all sections 13-20
</commit_message>
<xml_diff>
--- a/CSE Class Routine Fall-2026 (1).xlsx
+++ b/CSE Class Routine Fall-2026 (1).xlsx
@@ -203,7 +203,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="18">
     <border/>
     <border>
       <left style="thin">
@@ -349,11 +349,24 @@
       </top>
       <bottom/>
     </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+      <bottom style="thin">
+        <color rgb="FF999999"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="FF999999"/>
+      </right>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -556,6 +569,7 @@
     <xf numFmtId="0" fontId="2" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2246,8 +2260,15 @@
 RBS | 902</t>
         </is>
       </c>
-      <c r="G32" s="64" t="n"/>
-      <c r="H32" s="20" t="n"/>
+      <c r="G32" s="74" t="inlineStr">
+        <is>
+          <t>CSE 4148
+Mobile Application Development
+3:30-5:00
+RBS | 902</t>
+        </is>
+      </c>
+      <c r="H32" s="74" t="n"/>
       <c r="I32" s="2" t="n"/>
       <c r="J32" s="2" t="n"/>
       <c r="K32" s="2" t="n"/>
@@ -2445,7 +2466,7 @@
         <is>
           <t>CSE 3131
 Data Communication &amp; Networking
-3:30-5:00
+1:00-2:30
 TH | 804</t>
         </is>
       </c>
@@ -3716,15 +3737,17 @@
       <c r="D65" s="12" t="n"/>
       <c r="E65" s="31" t="inlineStr">
         <is>
+          <t>Jumu'ah Break</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
           <t>EEE 1212
 Electrical Circuit Analysis +  Lab
 2:30-5:00
 MES | 1503</t>
         </is>
       </c>
-      <c r="F65" s="64" t="n"/>
-      <c r="G65" s="2" t="n"/>
-      <c r="H65" s="2" t="n"/>
       <c r="I65" s="2" t="n"/>
       <c r="J65" s="2" t="n"/>
       <c r="K65" s="2" t="n"/>
@@ -3881,7 +3904,7 @@
         <is>
           <t>HUM 3103 *
 Principles of Management
-1:00-2:30
+2:30-4:00
 RH | 801</t>
         </is>
       </c>
@@ -4382,7 +4405,7 @@
         <is>
           <t>CSE 1111
 Theory of Computing
-9:00-10:30
+2:30-4:00
 MAR | 803</t>
         </is>
       </c>
@@ -8215,7 +8238,14 @@
 ASMS | 1101</t>
         </is>
       </c>
-      <c r="C169" s="64" t="n"/>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>CSE 1203
+Discrete Mathematics
+10:30 - 12:00
+IJ | 1101</t>
+        </is>
+      </c>
       <c r="D169" s="9" t="inlineStr">
         <is>
           <t>Lunch Break</t>
@@ -8962,8 +8992,14 @@
 TA | 1701</t>
         </is>
       </c>
-      <c r="G186" s="66" t="n"/>
-      <c r="H186" s="64" t="n"/>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>MATH 1111
+Mathematics-I
+3:30-5:00
+TA | 1701</t>
+        </is>
+      </c>
       <c r="I186" s="2" t="n"/>
       <c r="J186" s="2" t="n"/>
       <c r="K186" s="2" t="n"/>
@@ -9112,7 +9148,7 @@
         <is>
           <t>MATH 1111
 Mathematics-I
-2:30-4:00
+1:00-2:30
 TA | 1701</t>
         </is>
       </c>
@@ -9120,7 +9156,7 @@
         <is>
           <t>CSE 1213
 Structured Programming Language
-10:30 - 12:00
+2:30-4:00
 TBA | 1701</t>
         </is>
       </c>
@@ -9233,7 +9269,7 @@
         <is>
           <t>CSE 1213
 Structured Programming Language
-2:30-4:00
+1:00-2:30
 TBA | 801</t>
         </is>
       </c>
@@ -32127,7 +32163,7 @@
       <c r="Z1000" s="2" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="106">
+  <mergeCells count="105">
     <mergeCell ref="B91:C91"/>
     <mergeCell ref="E139:F139"/>
     <mergeCell ref="B40:H40"/>
@@ -32142,7 +32178,6 @@
     <mergeCell ref="B61:C61"/>
     <mergeCell ref="B194:H194"/>
     <mergeCell ref="A133:H133"/>
-    <mergeCell ref="E65:F65"/>
     <mergeCell ref="B184:H184"/>
     <mergeCell ref="B69:C69"/>
     <mergeCell ref="B38:C38"/>
@@ -32152,6 +32187,7 @@
     <mergeCell ref="E49:F49"/>
     <mergeCell ref="B195:H195"/>
     <mergeCell ref="E116:F116"/>
+    <mergeCell ref="F65:H65"/>
     <mergeCell ref="E136:F136"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="B172:H172"/>
@@ -32180,7 +32216,6 @@
     <mergeCell ref="B162:H162"/>
     <mergeCell ref="A199:H199"/>
     <mergeCell ref="B160:C160"/>
-    <mergeCell ref="B169:C169"/>
     <mergeCell ref="B19:H19"/>
     <mergeCell ref="B54:C54"/>
     <mergeCell ref="B74:H74"/>
@@ -32194,7 +32229,7 @@
     <mergeCell ref="B120:C120"/>
     <mergeCell ref="A177:H177"/>
     <mergeCell ref="F43:H43"/>
-    <mergeCell ref="F186:H186"/>
+    <mergeCell ref="G186:H186"/>
     <mergeCell ref="G87:H87"/>
     <mergeCell ref="A56:H56"/>
     <mergeCell ref="B171:C171"/>
@@ -32207,6 +32242,7 @@
     <mergeCell ref="G54:H54"/>
     <mergeCell ref="E72:F72"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="G32:H32"/>
     <mergeCell ref="B73:H73"/>
     <mergeCell ref="A111:H111"/>
     <mergeCell ref="A34:H34"/>
@@ -32222,7 +32258,6 @@
     <mergeCell ref="A78:H78"/>
     <mergeCell ref="B206:H206"/>
     <mergeCell ref="E182:F182"/>
-    <mergeCell ref="F32:G32"/>
     <mergeCell ref="A89:H89"/>
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="B87:C87"/>

</xml_diff>